<commit_message>
Final fase 3 requerimiento
</commit_message>
<xml_diff>
--- a/docs/importantes/Acta de reunion ciclo 1.xlsx
+++ b/docs/importantes/Acta de reunion ciclo 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e03e2c4a614451c2/Documentos/Bitacoras/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\pryectos print(nul)\docs\importantes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{F829444C-2C9B-41BB-87A9-E68B081804F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A8182FE5-8A31-4E49-A2EF-C0F6C8F149FE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664DFA58-B0D5-49E5-8824-F9DCFD4B2F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>Acta de Reuniones</t>
   </si>
@@ -104,13 +105,31 @@
   <si>
     <t>Revision grupal de los documentos que se repartieron en la tercera reunion 
 (administracion de configuraciones, plan de riesgos y definicion de estrategias)</t>
+  </si>
+  <si>
+    <t>Documentacion Script de
+ requerimientos y asignacion casos de uso</t>
+  </si>
+  <si>
+    <t>se realizo la reunion grupal con el objetivo de diligenciar el script de requerimientos y establecer los casos
+de uso para el proyecto, al mismo tiempo repartimos los casos de uso y escenarios de calidad para que cada 
+integrante se encargue de un tema en especifico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Realización de modelo de casos de uso </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se realizo en equipo el modelo de casos de uso, utilizando las especificaciones de casos de uso que se asigno a cada integrante </t>
+  </si>
+  <si>
+    <t>Revision grupal de los documentos que se repartieron, atributos de calidad y etc</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -550,21 +569,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9829B68-FADE-49C4-8C01-738BC2C2AD6B}">
-  <dimension ref="B1:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:M10"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="2" width="11.5546875" style="1"/>
-    <col min="3" max="3" width="9.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5546875" style="1"/>
-    <col min="5" max="5" width="7.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="92.33203125" style="1" customWidth="1"/>
-    <col min="8" max="12" width="11.5546875" style="1"/>
+    <col min="1" max="2" width="11.5" style="1"/>
+    <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5" style="1"/>
+    <col min="5" max="5" width="7.875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="92.375" style="1" customWidth="1"/>
+    <col min="8" max="12" width="11.5" style="1"/>
     <col min="13" max="13" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.5546875" style="1"/>
+    <col min="14" max="16384" width="11.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:13">
       <c r="B1" s="9" t="s">
         <v>0</v>
       </c>
@@ -580,7 +599,7 @@
       <c r="L1" s="9"/>
       <c r="M1" s="9"/>
     </row>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13">
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
@@ -594,7 +613,7 @@
       <c r="L2" s="9"/>
       <c r="M2" s="9"/>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" ht="15">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
@@ -632,7 +651,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:13" ht="28.5">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -658,7 +677,7 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" ht="28.5">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -684,7 +703,7 @@
       <c r="L5" s="8"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" ht="42.75">
       <c r="B6" s="3">
         <v>3</v>
       </c>
@@ -710,7 +729,7 @@
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
     </row>
-    <row r="7" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" ht="28.5">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -736,37 +755,83 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" ht="42.75">
       <c r="B8" s="3">
         <v>5</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="M8" s="3"/>
-    </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="C8" s="4">
+        <v>45897</v>
+      </c>
+      <c r="D8" s="5">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="E8" s="5">
+        <v>0.89583333333333337</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="7"/>
+    </row>
+    <row r="9" spans="2:13" ht="28.5">
       <c r="B9" s="3">
         <v>6</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
+      <c r="C9" s="4">
+        <v>45902</v>
+      </c>
+      <c r="D9" s="5">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
+      <c r="J9" s="7"/>
+      <c r="K9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="7"/>
+    </row>
+    <row r="10" spans="2:13">
+      <c r="B10" s="3">
+        <v>7</v>
+      </c>
+      <c r="C10" s="4">
+        <v>45902</v>
+      </c>
+      <c r="D10" s="5">
+        <v>0.9375</v>
+      </c>
+      <c r="E10" s="5">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Final fase 4 planeacion
</commit_message>
<xml_diff>
--- a/docs/importantes/Acta de reunion ciclo 1.xlsx
+++ b/docs/importantes/Acta de reunion ciclo 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\pryectos print(nul)\docs\importantes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{664DFA58-B0D5-49E5-8824-F9DCFD4B2F94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF57FD0-6C9A-4088-B11B-7D059B45A7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
   <si>
     <t>Acta de Reuniones</t>
   </si>
@@ -123,6 +123,17 @@
   </si>
   <si>
     <t>Revision grupal de los documentos que se repartieron, atributos de calidad y etc</t>
+  </si>
+  <si>
+    <t>diligenciar script de procesos (planecion)</t>
+  </si>
+  <si>
+    <t>Sese realizo la reunion grupal con la intencion de diligenciar el script de procesos enfocado a la
+fase de planeacion del proyecto, donde se distribuyeron los diferentes documentos relacionados a la entrega
+de planeacion</t>
+  </si>
+  <si>
+    <t>Revision grupal de los documentos plan de requerimientos, plan de calidad y EDT</t>
   </si>
 </sst>
 </file>
@@ -246,10 +257,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -569,14 +576,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9829B68-FADE-49C4-8C01-738BC2C2AD6B}">
-  <dimension ref="B1:M10"/>
+  <dimension ref="B1:M12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="2" width="11.5" style="1"/>
     <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.5" style="1"/>
+    <col min="4" max="4" width="10" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="32.75" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="34.125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="92.375" style="1" customWidth="1"/>
     <col min="8" max="12" width="11.5" style="1"/>
     <col min="13" max="13" width="13" style="1" bestFit="1" customWidth="1"/>
@@ -833,6 +840,58 @@
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
     </row>
+    <row r="11" spans="2:13" ht="42.75">
+      <c r="B11" s="3">
+        <v>8</v>
+      </c>
+      <c r="C11" s="4">
+        <v>45904</v>
+      </c>
+      <c r="D11" s="5">
+        <v>0.75</v>
+      </c>
+      <c r="E11" s="5">
+        <v>0.875</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="7"/>
+    </row>
+    <row r="12" spans="2:13">
+      <c r="B12" s="3">
+        <v>9</v>
+      </c>
+      <c r="C12" s="4">
+        <v>45908</v>
+      </c>
+      <c r="D12" s="5">
+        <v>0.9375</v>
+      </c>
+      <c r="E12" s="5">
+        <v>0.97916666666666663</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="7"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B1:M2"/>

</xml_diff>

<commit_message>
Final fase 5 diseño
</commit_message>
<xml_diff>
--- a/docs/importantes/Acta de reunion ciclo 1.xlsx
+++ b/docs/importantes/Acta de reunion ciclo 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\pryectos print(nul)\docs\importantes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\esteb\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFF57FD0-6C9A-4088-B11B-7D059B45A7E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C9B8178-87B2-4D26-8406-AC27775F2479}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{62DC227A-B2C0-4B2D-82A6-53B37F2213DD}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -29,15 +29,12 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="28">
   <si>
     <t>Acta de Reuniones</t>
   </si>
@@ -125,22 +122,18 @@
     <t>Revision grupal de los documentos que se repartieron, atributos de calidad y etc</t>
   </si>
   <si>
-    <t>diligenciar script de procesos (planecion)</t>
-  </si>
-  <si>
-    <t>Sese realizo la reunion grupal con la intencion de diligenciar el script de procesos enfocado a la
-fase de planeacion del proyecto, donde se distribuyeron los diferentes documentos relacionados a la entrega
-de planeacion</t>
-  </si>
-  <si>
-    <t>Revision grupal de los documentos plan de requerimientos, plan de calidad y EDT</t>
+    <t>Documentacion Script de
+ requerimientos y asignacion diagramas UML</t>
+  </si>
+  <si>
+    <t>Se realizo la reunion con el objetivo de coordinar y dejar todos diagramas UML y las diferentes partes de el documento entregable divididas entre los miembros del equipo</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,7 +159,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -176,12 +169,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -213,7 +200,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -234,9 +221,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -576,51 +560,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9829B68-FADE-49C4-8C01-738BC2C2AD6B}">
-  <dimension ref="B1:M12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="14.25"/>
+  <dimension ref="B1:M11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="11.5" style="1"/>
-    <col min="3" max="3" width="10.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="34.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="92.375" style="1" customWidth="1"/>
-    <col min="8" max="12" width="11.5" style="1"/>
+    <col min="1" max="2" width="11.44140625" style="1"/>
+    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.44140625" style="1"/>
+    <col min="5" max="5" width="7.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="32.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="92.33203125" style="1" customWidth="1"/>
+    <col min="8" max="12" width="11.44140625" style="1"/>
     <col min="13" max="13" width="13" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="11.5" style="1"/>
+    <col min="14" max="16384" width="11.44140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:13">
-      <c r="B1" s="9" t="s">
+    <row r="1" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="9"/>
-    </row>
-    <row r="2" spans="2:13">
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
-    </row>
-    <row r="3" spans="2:13" ht="15">
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+    </row>
+    <row r="2" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+    </row>
+    <row r="3" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
@@ -658,7 +642,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="28.5">
+    <row r="4" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="3">
         <v>1</v>
       </c>
@@ -684,7 +668,7 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="2:13" ht="28.5">
+    <row r="5" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B5" s="3">
         <v>2</v>
       </c>
@@ -707,10 +691,10 @@
       <c r="I5" s="7"/>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
-      <c r="L5" s="8"/>
+      <c r="L5" s="7"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="2:13" ht="42.75">
+    <row r="6" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B6" s="3">
         <v>3</v>
       </c>
@@ -736,7 +720,7 @@
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
     </row>
-    <row r="7" spans="2:13" ht="28.5">
+    <row r="7" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B7" s="3">
         <v>4</v>
       </c>
@@ -762,7 +746,7 @@
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
     </row>
-    <row r="8" spans="2:13" ht="42.75">
+    <row r="8" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="3">
         <v>5</v>
       </c>
@@ -788,7 +772,7 @@
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
     </row>
-    <row r="9" spans="2:13" ht="28.5">
+    <row r="9" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B9" s="3">
         <v>6</v>
       </c>
@@ -814,7 +798,7 @@
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
     </row>
-    <row r="10" spans="2:13">
+    <row r="10" spans="2:13" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
         <v>7</v>
       </c>
@@ -840,20 +824,20 @@
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
     </row>
-    <row r="11" spans="2:13" ht="42.75">
+    <row r="11" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
         <v>8</v>
       </c>
       <c r="C11" s="4">
-        <v>45904</v>
+        <v>45915</v>
       </c>
       <c r="D11" s="5">
-        <v>0.75</v>
+        <v>0.79166666666666663</v>
       </c>
       <c r="E11" s="5">
-        <v>0.875</v>
-      </c>
-      <c r="F11" s="3" t="s">
+        <v>0.85416666666666663</v>
+      </c>
+      <c r="F11" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="6" t="s">
@@ -865,32 +849,6 @@
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
-    </row>
-    <row r="12" spans="2:13">
-      <c r="B12" s="3">
-        <v>9</v>
-      </c>
-      <c r="C12" s="4">
-        <v>45908</v>
-      </c>
-      <c r="D12" s="5">
-        <v>0.9375</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0.97916666666666663</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>